<commit_message>
Corrige gerador da BOM: itens eliminados voltavam para a lista de compras
A tabela "Itens que NAO existem mais nesta versao" tem "Item removido"
no cabecalho, e o filtro so testava "Item" — entao ela era importada
como se fossem itens a comprar. Alem disso, o guard contra tachado
(~~item~~) rodava DEPOIS de limpar(), que ja havia removido os "~~",
entao nunca disparava.

Resultado: XL4016, XL4015, 6 diodos Zener, cooler de 30 mm, tubo de
63 mm e os voltimetros de 3 fios apareciam na planilha de compras.

Correcoes:
- checagem de tachado feita na celula BRUTA, antes de limpar()
- secoes de itens removidos ignoradas por regex

Planilha regerada: 166 itens em 17 secoes (era 182 em 18, com 16 itens
fantasmas). Aba "Dados do Projeto" atualizada com os numeros da
arquitetura "Potencia em 24 V".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM_Projeto_Integrador.xlsx
+++ b/BOM_Projeto_Integrador.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Dados do Projeto" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista de Compras'!$A$4:$H$188</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista de Compras'!$A$4:$H$187</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -574,7 +574,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lista de materiais · gerada de 03_lista_materiais.md em 12/08/2026 22:07 · arquitetura 127 V CA → 24 V CC → 12 / 5 / 3,3 V</t>
+          <t>Lista de materiais · gerada de 03_lista_materiais.md em 13/08/2026 19:12 · arquitetura 127 V CA → 24 V CC → 12 / 5 / 3,3 V</t>
         </is>
       </c>
     </row>
@@ -888,22 +888,22 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>T1 — Módulo XL4016</t>
+          <t>⭐ Kit 2× Módulo LM2596 com display</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1 kit</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>Step-down 8 A / 300 W, CC+CV, Vin 8-40 V</t>
+          <t>Step-down 3 A, Vin até 40 V, saída ajustável, display LED vermelho de 3 dígitos integrado. Um módulo vira o T2, o outro vira o T3</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>12,0 V / 7,0 A</t>
+          <t>ver abaixo</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr"/>
@@ -919,22 +919,22 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>T2 — Módulo XL4015</t>
+          <t>→ T2 (poste P2, comando)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Step-down 5 A, CC+CV (o do seu link)</t>
+          <t>1º módulo do kit — alimenta Arduino, Nextion, SD/RTC, lógica dos BTS, placa PI-1 e os LEDs da iluminação da maquete</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>5,10 V / 1,5 A</t>
+          <t>5,10 V</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr"/>
@@ -950,22 +950,22 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>T3 — Módulo XL4015</t>
+          <t>→ T3 (poste P3, auxiliares)</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Step-down 5 A, CC+CV (o do seu link)</t>
+          <t>2º módulo do kit — alimenta as fans internas e os coolers</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>12,0 V / 1,5 A</t>
+          <t>12,0 V</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr"/>
@@ -981,17 +981,17 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Dissipador de alumínio 40×40×20 mm</t>
+          <t>Kit LM2596 reserva</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1 kit</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Colado com fita térmica no CI e no diodo de cada módulo</t>
+          <t>Opcional mas recomendado. São os únicos conversores do projeto; queimar um na véspera sem reserva significa não apresentar</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -1012,17 +1012,17 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Fita térmica dupla face</t>
+          <t>Dissipador de alumínio ~20 × 15 × 10 mm</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Fixação dos dissipadores</t>
+          <t>⚠️ Obrigatório, colado no CI LM2596S de cada módulo. Sem ele o T3 passa dos 100 °C dentro do tubo — ver Doc 02 §2.8</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Voltímetro digital 3 fios (0-100 V)</t>
+          <t>Fita térmica dupla face</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Leitor na frente do T2 e do T3. ⚠️ 3 fios (alimentação separada): o de 2 fios não lê 5,10 V de forma estável</t>
+          <t>Fixação dos dissipadores</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1074,17 +1074,17 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Voltímetro + amperímetro digital 3 fios</t>
+          <t>Acrílico transparente 1 mm</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1 lâmina</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Leitor na frente do T1 — mostra 12,0 V e a corrente da Peltier ao vivo</t>
+          <t>Janelas de visualização nos 3 tubos dos postes (~20 × 12 mm cada) — protege o display e mantém o visual fechado</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Acrílico 1 mm</t>
+          <t>Voltímetro + amperímetro digital 3 fios</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Janelinha de proteção dos 3 leitores</t>
+          <t>Único medidor comprado à parte — vai na caixa de derivação do P1, mostrando os 24,0 V do barramento e a corrente das Peltier ao vivo. Faixa: 0-100 V / 10 A</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>F1, F2, F3, F4, F5</t>
+          <t>F1, F2, F3 — entrada dos 3 ramais</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr"/>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Fusível mini automotivo 6 A</t>
+          <t>Fusível mini automotivo 10 A</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>F1 — ramal R1 (potência)</t>
+          <t>F1 — ramal R1 (potência 24 V, 6,0 A)</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr"/>
@@ -1210,17 +1210,17 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>3 usos + reservas</t>
+          <t>2 usos + 2 reservas</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>F2, F3 (ramais) e F4 (saída 5 V)</t>
+          <t>F2 (comando) e F3 (auxiliares)</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr"/>
@@ -1236,22 +1236,22 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Fusível mini automotivo 10 A</t>
+          <t>Terminal olhal M4 amarelo</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>1 uso + 1 reserva</t>
+          <t>Aterramento e barramento de 0 V</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>F5 — saída 12 V dos BTS</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr"/>
@@ -1261,61 +1261,33 @@
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Diodo Zener 5V6 / 5 W</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Crowbar de proteção do barramento 5 V</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Saída do T2</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr"/>
-      <c r="G28" s="8" t="inlineStr"/>
-      <c r="H28" s="8">
-        <f>IF(C28*G28=0,"",C28*G28)</f>
-        <v/>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>M.1 — Base e estrutura</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Diodo Zener 13 V / 5 W</t>
+          <t>MDF 12 mm</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1 chapa</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Crowbar do barramento 12 V auxiliar</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>Saída do T3</t>
-        </is>
-      </c>
+          <t>1500 × 500 mm — tampo da base</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr"/>
       <c r="F29" s="11" t="inlineStr"/>
       <c r="G29" s="12" t="inlineStr"/>
       <c r="H29" s="12">
@@ -1325,28 +1297,24 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Diodo Zener 15 V / 5 W</t>
+          <t>MDF 15 mm</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Crowbar do barramento 12 V de potência</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Saída do T1</t>
-        </is>
-      </c>
+          <t>Moldura perimetral 40 mm de altura (4 tiras)</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr"/>
       <c r="F30" s="7" t="inlineStr"/>
       <c r="G30" s="8" t="inlineStr"/>
       <c r="H30" s="8">
@@ -1356,28 +1324,24 @@
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Terminal olhal M4 amarelo</t>
+          <t>MDF 15 mm</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3 tiras</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Aterramento e barramento de 0 V</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>Travessas de reforço 15 × 40 mm, com entalhe de 20 × 25 mm no centro</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr"/>
       <c r="F31" s="11" t="inlineStr"/>
       <c r="G31" s="12" t="inlineStr"/>
       <c r="H31" s="12">
@@ -1385,11 +1349,31 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>M.1 — Base e estrutura</t>
-        </is>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Pés de borracha antiderrapante</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Autoadesivos, Ø 25 mm — a base tem 1,5 m e pesa ~18 kg</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr"/>
+      <c r="F32" s="7" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr"/>
+      <c r="H32" s="8">
+        <f>IF(C32*G32=0,"",C32*G32)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -1398,17 +1382,17 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>MDF 12 mm</t>
+          <t>Conector circular GX16 8 pinos</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>1 chapa</t>
+          <t>1 par</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>1500 × 500 mm — tampo da base</t>
+          <t>Opcional — só na versão modular (união elétrica entre os 2 módulos)</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr"/>
@@ -1425,17 +1409,17 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>MDF 15 mm</t>
+          <t>Pinos-guia Ø 6 mm + buchas</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Moldura perimetral 40 mm de altura (4 tiras)</t>
+          <t>Opcional — alinhamento dos módulos</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr"/>
@@ -1452,17 +1436,17 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>MDF 15 mm</t>
+          <t>Alças de transporte</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>3 tiras</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>Travessas de reforço 15 × 40 mm, com entalhe de 20 × 25 mm no centro</t>
+          <t>Alça embutida de baú/case, laterais</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr"/>
@@ -1479,17 +1463,17 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Pés de borracha antiderrapante</t>
+          <t>Parafusos M5×20, M4×16, M3×12</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>kits</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Autoadesivos, Ø 25 mm — a base tem 1,5 m e pesa ~18 kg</t>
+          <t>Fixações gerais</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr"/>
@@ -1506,17 +1490,17 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Conector circular GX16 8 pinos</t>
+          <t>Insertos rosqueados M4/M5 p/ MDF</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>1 par</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>Opcional — só na versão modular (união elétrica entre os 2 módulos)</t>
+          <t>Evita espanar a rosca no MDF</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr"/>
@@ -1527,50 +1511,30 @@
         <v/>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>Pinos-guia Ø 6 mm + buchas</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>Opcional — alinhamento dos módulos</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="inlineStr"/>
-      <c r="F38" s="7" t="inlineStr"/>
-      <c r="G38" s="8" t="inlineStr"/>
-      <c r="H38" s="8">
-        <f>IF(C38*G38=0,"",C38*G38)</f>
-        <v/>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>M.2 — Subestação (caixa)</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Alças de transporte</t>
+          <t>MDF 9 mm ou acrílico opaco 4 mm</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Alça embutida de baú/case, laterais</t>
+          <t>Caixa 260 × 190 × 150 mm (L×P×A), frente voltada para a rua</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr"/>
@@ -1583,21 +1547,21 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Parafusos M5×20, M4×16, M3×12</t>
+          <t>Dobradiça pequena + fecho</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>kits</t>
+          <t>1 jogo</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Fixações gerais</t>
+          <t>Tampa de manutenção</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr"/>
@@ -1610,21 +1574,21 @@
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Insertos rosqueados M4/M5 p/ MDF</t>
+          <t>Tela metálica / alambrado miniatura</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Evita espanar a rosca no MDF</t>
+          <t>Cerca do pátio da subestação (tela de aço, malha 3 mm)</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr"/>
@@ -1635,11 +1599,31 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>M.2 — Subestação (caixa)</t>
-        </is>
+    <row r="42">
+      <c r="A42" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Pedrisco / brita fina (aquário)</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>500 g</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Piso do pátio da subestação — como nas subestações reais</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr"/>
+      <c r="F42" s="7" t="inlineStr"/>
+      <c r="G42" s="8" t="inlineStr"/>
+      <c r="H42" s="8">
+        <f>IF(C42*G42=0,"",C42*G42)</f>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -1648,17 +1632,17 @@
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>MDF 9 mm ou acrílico opaco 4 mm</t>
+          <t>Placa "PERIGO ALTA TENSÃO"</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>Caixa 260 × 190 × 150 mm (L×P×A), frente voltada para a rua</t>
+          <t>Impressa em papel adesivo, ~15 × 10 mm</t>
         </is>
       </c>
       <c r="E43" s="10" t="inlineStr"/>
@@ -1669,50 +1653,30 @@
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="n">
-        <v>35</v>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>Dobradiça pequena + fecho</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>1 jogo</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>Tampa de manutenção</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr"/>
-      <c r="F44" s="7" t="inlineStr"/>
-      <c r="G44" s="8" t="inlineStr"/>
-      <c r="H44" s="8">
-        <f>IF(C44*G44=0,"",C44*G44)</f>
-        <v/>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>M.3 — Postes e linha de distribuição</t>
+        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Tela metálica / alambrado miniatura</t>
+          <t>Tubo de alumínio Ø 8 mm</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1,5 m</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>Cerca do pátio da subestação (tela de aço, malha 3 mm)</t>
+          <t>Cortar em 3 postes de 350 mm (300 mm visíveis + 50 mm de encaixe)</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr"/>
@@ -1725,21 +1689,21 @@
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Pedrisco / brita fina (aquário)</t>
+          <t>Barra chata de alumínio 12 × 2 mm</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>500 g</t>
+          <t>40 cm</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>Piso do pátio da subestação — como nas subestações reais</t>
+          <t>Cruzetas — 3 peças de 90 mm + 3 de 60 mm</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr"/>
@@ -1752,21 +1716,21 @@
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Placa "PERIGO ALTA TENSÃO"</t>
+          <t>Fio rígido ENCAPADO 1,00 mm² VERMELHO ⬆</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2 m</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>Impressa em papel adesivo, ~15 × 10 mm</t>
+          <t>Ramal R1 (potência, 6,0 A). ⚠️ Subiu de 0,75 para 1,00 mm² por causa da corrente das 2 Peltier. Nunca condutor nu — em CC qualquer ponte metálica é curto franco</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr"/>
@@ -1777,11 +1741,31 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>M.3 — Postes e linha de distribuição</t>
-        </is>
+    <row r="48">
+      <c r="A48" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Fio rígido ENCAPADO 0,50 mm² MARROM</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Ramal R2 (comando)</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr"/>
+      <c r="F48" s="7" t="inlineStr"/>
+      <c r="G48" s="8" t="inlineStr"/>
+      <c r="H48" s="8">
+        <f>IF(C48*G48=0,"",C48*G48)</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -1790,17 +1774,17 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Tubo de alumínio Ø 8 mm</t>
+          <t>Fio rígido ENCAPADO 0,50 mm² CINZA</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>1,5 m</t>
+          <t>2 m</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>Cortar em 3 postes de 350 mm (300 mm visíveis + 50 mm de encaixe)</t>
+          <t>Ramal R3 (auxiliares)</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr"/>
@@ -1817,17 +1801,17 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Barra chata de alumínio 12 × 2 mm</t>
+          <t>Fio rígido ENCAPADO 1,50 mm² AZUL CLARO ⬆</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>40 cm</t>
+          <t>2 m</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Cruzetas — 3 peças de 90 mm + 3 de 60 mm</t>
+          <t>Retorno comum 0 V — o "neutro" da linha, 40 mm abaixo da cruzeta. Subiu de 1,00 para 1,50 mm²: conduz a soma dos 3 ramais (6,9 A)</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr"/>
@@ -1844,17 +1828,17 @@
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Fio rígido ENCAPADO 0,75 mm² VERMELHO</t>
+          <t>Contas/miçangas marrom ou branca Ø 6 mm</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>Ramal R1 (potência). ⚠️ Nunca condutor nu — em CC qualquer ponte metálica é curto franco</t>
+          <t>Isoladores de pino da cruzeta</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr"/>
@@ -1871,17 +1855,17 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Fio rígido ENCAPADO 0,50 mm² MARROM</t>
+          <t>Tubo de PVC Ø 50 mm</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>24 cm</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Ramal R2 (comando)</t>
+          <t>Corpos dos 3 postes — 8 cm cada: T2 (P2), T3 (P3) e a caixa de derivação (P1). Agora os três têm o mesmo diâmetro, porque o P1 deixou de ter conversor</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr"/>
@@ -1898,17 +1882,17 @@
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Fio rígido ENCAPADO 0,50 mm² CINZA</t>
+          <t>Tampa/cap PVC Ø 50 mm</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>Ramal R3 (auxiliares)</t>
+          <t>Tampas dos 3 corpos</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr"/>
@@ -1925,17 +1909,17 @@
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Fio rígido ENCAPADO 1,00 mm² AZUL CLARO</t>
+          <t>Cinta de alumínio 10 mm</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>1 m</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Retorno comum 0 V — o "neutro" da linha, 40 mm abaixo da cruzeta</t>
+          <t>Fixação dos transformadores e da caixa de derivação nos postes</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr"/>
@@ -1952,17 +1936,17 @@
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Contas/miçangas marrom ou branca Ø 6 mm</t>
+          <t>Bornes de emenda pequenos (2 ou 3 vias)</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>Isoladores de pino da cruzeta</t>
+          <t>Dentro da caixa de derivação do P1 — ali os 24 V só se distribuem, não se transformam</t>
         </is>
       </c>
       <c r="E55" s="10" t="inlineStr"/>
@@ -1979,17 +1963,17 @@
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Tubo de PVC Ø 63 mm</t>
+          <t>Flange/base de fixação dos postes</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>10 cm</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Corpo do transformador T1 (maior — comporta o XL4016 + cooler)</t>
+          <t>Podem ser feitas com sobra de MDF + insertos M4</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr"/>
@@ -2006,17 +1990,17 @@
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Tubo de PVC Ø 50 mm</t>
+          <t>Etiquetas adesivas impressas</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>16 cm</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>Corpo dos transformadores T2 e T3</t>
+          <t>Identificação dos corpos: "P1 — DERIVAÇÃO 24 V", "T2 — 24/5 V", "T3 — 24/12 V"</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr"/>
@@ -2027,50 +2011,30 @@
         <v/>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="5" t="n">
-        <v>48</v>
-      </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>Tampa/cap PVC Ø 63 mm</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>Tampas do T1</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr"/>
-      <c r="F58" s="7" t="inlineStr"/>
-      <c r="G58" s="8" t="inlineStr"/>
-      <c r="H58" s="8">
-        <f>IF(C58*G58=0,"",C58*G58)</f>
-        <v/>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>M.4 — Rua e entrada da empresa (zona externa)</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Tampa/cap PVC Ø 50 mm</t>
+          <t>Tinta spray cinza-asfalto escuro fosco</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>Tampas do T2 e T3</t>
+          <t>Pista da rua</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr"/>
@@ -2083,21 +2047,21 @@
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Cooler 30 mm 12 V</t>
+          <t>Tubo de alumínio Ø 5 mm</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>60 cm</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Ventilação forçada dentro do T1 (dissipa ~10 W)</t>
+          <t>3 postes de iluminação pública de 180 mm — ⚠️ diferentes dos postes de distribuição</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr"/>
@@ -2110,11 +2074,11 @@
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Cinta de alumínio 10 mm</t>
+          <t>Arame 1,5 mm</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
@@ -2124,7 +2088,7 @@
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>Fixação dos transformadores nos postes</t>
+          <t>Braço curvo das luminárias e estrutura do portão</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr"/>
@@ -2137,21 +2101,21 @@
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Flange/base de fixação dos postes</t>
+          <t>LED 3 mm branco quente</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Podem ser feitas com sobra de MDF + insertos M4</t>
+          <t>3 luminárias da rua + 1 na guarita. Alimentados em 5 V (BD-5V), com 220 Ω em série, sempre acesos. Vf ≈ 3,1 V</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr"/>
@@ -2162,11 +2126,31 @@
         <v/>
       </c>
     </row>
-    <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t>M.4 — Rua e entrada da empresa (zona externa)</t>
-        </is>
+    <row r="63">
+      <c r="A63" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>Resistor 220 Ω 1/4 W</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
+        <is>
+          <t>Limitador dos LEDs da rua — já contabilizado na lista L.4, não compre de novo. ⚠️ Valor dimensionado para 5 V: (5 − 3,1)/220 = 8,6 mA. Monte cada um dentro da base do poste, com termorretrátil</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="inlineStr"/>
+      <c r="F63" s="11" t="inlineStr"/>
+      <c r="G63" s="12" t="inlineStr"/>
+      <c r="H63" s="12">
+        <f>IF(C63*G63=0,"",C63*G63)</f>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -2175,17 +2159,17 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Tinta spray cinza-asfalto escuro fosco</t>
+          <t>Carro de passeio miniatura 1:50</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Pista da rua</t>
+          <t>~88 mm. Se só achar 1:64 (68 mm), pode usar — mas não misture escalas</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr"/>
@@ -2202,17 +2186,17 @@
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Tubo de alumínio Ø 5 mm</t>
+          <t>Caminhão / van 1:50</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>60 cm</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>3 postes de iluminação pública de 180 mm — ⚠️ diferentes dos postes de distribuição</t>
+          <t>~150 mm, entrando pelo portão</t>
         </is>
       </c>
       <c r="E65" s="10" t="inlineStr"/>
@@ -2229,17 +2213,17 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Arame 1,5 mm</t>
+          <t>Tira de MDF 3 mm</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>1 m</t>
+          <t>1,5 m</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Braço curvo das luminárias e estrutura do portão</t>
+          <t>Meio-fio (guia), 4 mm de altura, pintado de branco</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr"/>
@@ -2256,17 +2240,17 @@
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>LED 3 mm branco quente</t>
+          <t>Fita branca 2 mm ou caneta posca branca</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>3 luminárias da rua + 1 na guarita</t>
+          <t>Faixa central tracejada, faixa de bordo e faixa de pedestres</t>
         </is>
       </c>
       <c r="E67" s="10" t="inlineStr"/>
@@ -2283,17 +2267,17 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Resistor 2,2 kΩ 1/4 W</t>
+          <t>MDF 4 mm</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>Limitador dos LEDs (24 V)</t>
+          <t>Muro da empresa: 50 mm de altura × 290 mm, em X = 640</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr"/>
@@ -2310,17 +2294,17 @@
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Carro de passeio miniatura 1:50</t>
+          <t>MDF 4 mm</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>~88 mm. Se só achar 1:64 (68 mm), pode usar — mas não misture escalas</t>
+          <t>Guarita 45 × 45 × 55 mm, com janela recortada</t>
         </is>
       </c>
       <c r="E69" s="10" t="inlineStr"/>
@@ -2337,7 +2321,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Caminhão / van 1:50</t>
+          <t>Tinta azul industrial</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
@@ -2347,7 +2331,7 @@
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>~150 mm, entrando pelo portão</t>
+          <t>Portão corrediço</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr"/>
@@ -2364,17 +2348,17 @@
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Tira de MDF 3 mm</t>
+          <t>Árvores de maquete</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>1,5 m</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>Meio-fio (guia), 4 mm de altura, pintado de branco</t>
+          <t>Escala 1:50, na calçada da frente</t>
         </is>
       </c>
       <c r="E71" s="10" t="inlineStr"/>
@@ -2391,17 +2375,17 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Fita branca 2 mm ou caneta posca branca</t>
+          <t>Placas de trânsito miniatura</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>Faixa central tracejada, faixa de bordo e faixa de pedestres</t>
+          <t>"PARE" e "VELOCIDADE MÁXIMA 10 km/h"</t>
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr"/>
@@ -2418,17 +2402,17 @@
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>MDF 4 mm</t>
+          <t>Lixeira urbana + abrigo de ônibus</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1 cada</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>Muro da empresa: 50 mm de altura × 290 mm, em X = 640</t>
+          <t>Opcional — enriquece a cena</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr"/>
@@ -2439,50 +2423,30 @@
         <v/>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="5" t="n">
-        <v>63</v>
-      </c>
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>MDF 4 mm</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>Guarita 45 × 45 × 55 mm, com janela recortada</t>
-        </is>
-      </c>
-      <c r="E74" s="6" t="inlineStr"/>
-      <c r="F74" s="7" t="inlineStr"/>
-      <c r="G74" s="8" t="inlineStr"/>
-      <c r="H74" s="8">
-        <f>IF(C74*G74=0,"",C74*G74)</f>
-        <v/>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>M.5 — Chão de fábrica (cenografia)</t>
+        </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Tinta azul industrial</t>
+          <t>Tinta spray cinza claro fosco</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>Portão corrediço</t>
+          <t>Piso industrial (epóxi)</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr"/>
@@ -2495,21 +2459,21 @@
     </row>
     <row r="76">
       <c r="A76" s="5" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Árvores de maquete</t>
+          <t>Tinta spray preto fosco</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>Escala 1:50, na calçada da frente</t>
+          <t>Estruturas e acabamento</t>
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr"/>
@@ -2522,21 +2486,21 @@
     </row>
     <row r="77">
       <c r="A77" s="9" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>Placas de trânsito miniatura</t>
+          <t>Verniz fosco spray</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>"PARE" e "VELOCIDADE MÁXIMA 10 km/h"</t>
+          <t>Proteção final do piso pintado</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr"/>
@@ -2549,21 +2513,21 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>Lixeira urbana + abrigo de ônibus</t>
+          <t>Fita adesiva amarela 10 mm</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>1 cada</t>
+          <t>1 rolo</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>Opcional — enriquece a cena</t>
+          <t>Demarcação de corredores e áreas</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr"/>
@@ -2574,11 +2538,31 @@
         <v/>
       </c>
     </row>
-    <row r="79" ht="22" customHeight="1">
-      <c r="A79" s="4" t="inlineStr">
-        <is>
-          <t>M.5 — Chão de fábrica (cenografia)</t>
-        </is>
+    <row r="79">
+      <c r="A79" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t>Fita zebrada amarelo/preto 20 mm</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>1 rolo</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>Faixa de segurança em frente ao painel (exigência NR-10 — zona de trabalho)</t>
+        </is>
+      </c>
+      <c r="E79" s="10" t="inlineStr"/>
+      <c r="F79" s="11" t="inlineStr"/>
+      <c r="G79" s="12" t="inlineStr"/>
+      <c r="H79" s="12">
+        <f>IF(C79*G79=0,"",C79*G79)</f>
+        <v/>
       </c>
     </row>
     <row r="80">
@@ -2587,17 +2571,17 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>Tinta spray cinza claro fosco</t>
+          <t>Fita adesiva verde 10 mm</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1 rolo</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>Piso industrial (epóxi)</t>
+          <t>Rota de fuga</t>
         </is>
       </c>
       <c r="E80" s="6" t="inlineStr"/>
@@ -2614,17 +2598,17 @@
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Tinta spray preto fosco</t>
+          <t>Figuras de maquete escala 1:50</t>
         </is>
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>Estruturas e acabamento</t>
+          <t>(4 na fábrica, 3 na rua, 3 reservas) Pessoas com EPI (loja de maquetaria/arquitetura)</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr"/>
@@ -2641,17 +2625,17 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>Verniz fosco spray</t>
+          <t>Miniaturas: empilhadeira, pallets, tambores</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>Proteção final do piso pintado</t>
+          <t>Ambientação do chão de fábrica</t>
         </is>
       </c>
       <c r="E82" s="6" t="inlineStr"/>
@@ -2668,17 +2652,17 @@
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Fita adesiva amarela 10 mm</t>
+          <t>Extintor miniatura + placa</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>1 rolo</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>Demarcação de corredores e áreas</t>
+          <t>Sinalização de segurança</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr"/>
@@ -2695,17 +2679,17 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Fita zebrada amarelo/preto 20 mm</t>
+          <t>Placas de sinalização impressas</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>1 rolo</t>
+          <t>1 folha</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>Faixa de segurança em frente ao painel (exigência NR-10 — zona de trabalho)</t>
+          <t>"RISCO ELÉTRICO", "USO OBRIGATÓRIO DE EPI", "SAÍDA" — papel adesivo</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr"/>
@@ -2722,17 +2706,17 @@
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>Fita adesiva verde 10 mm</t>
+          <t>Eletrocalha / perfilado aéreo</t>
         </is>
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>1 rolo</t>
+          <t>60 cm</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>Rota de fuga</t>
+          <t>Canaleta de acrílico ou perfil U de alumínio — leva os cabos do painel à câmara por cima, como na indústria</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr"/>
@@ -2749,17 +2733,17 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>Figuras de maquete escala 1:50</t>
+          <t>Suportes/mãos-francesas da eletrocalha</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>(4 na fábrica, 3 na rua, 3 reservas) Pessoas com EPI (loja de maquetaria/arquitetura)</t>
+          <t>Cantoneira de alumínio</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr"/>
@@ -2776,7 +2760,7 @@
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>Miniaturas: empilhadeira, pallets, tambores</t>
+          <t>EVA ou MDF 6 mm</t>
         </is>
       </c>
       <c r="C87" s="9" t="inlineStr">
@@ -2786,7 +2770,7 @@
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t>Ambientação do chão de fábrica</t>
+          <t>Bases de máquinas fictícias e plataformas</t>
         </is>
       </c>
       <c r="E87" s="10" t="inlineStr"/>
@@ -2797,50 +2781,30 @@
         <v/>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="5" t="n">
-        <v>76</v>
-      </c>
-      <c r="B88" s="6" t="inlineStr">
-        <is>
-          <t>Extintor miniatura + placa</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D88" s="6" t="inlineStr">
-        <is>
-          <t>Sinalização de segurança</t>
-        </is>
-      </c>
-      <c r="E88" s="6" t="inlineStr"/>
-      <c r="F88" s="7" t="inlineStr"/>
-      <c r="G88" s="8" t="inlineStr"/>
-      <c r="H88" s="8">
-        <f>IF(C88*G88=0,"",C88*G88)</f>
-        <v/>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>C.2 — Isolamento térmico</t>
+        </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Placas de sinalização impressas</t>
+          <t>XPS 30 mm (poliestireno extrudado)</t>
         </is>
       </c>
       <c r="C89" s="9" t="inlineStr">
         <is>
-          <t>1 folha</t>
+          <t>1 m²</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>"RISCO ELÉTRICO", "USO OBRIGATÓRIO DE EPI", "SAÍDA" — papel adesivo</t>
+          <t>Isolante principal — k ≈ 0,033 W/m·K. 30 mm, não 20 mm (ver Doc 12)</t>
         </is>
       </c>
       <c r="E89" s="10" t="inlineStr"/>
@@ -2853,21 +2817,21 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>Eletrocalha / perfilado aéreo</t>
+          <t>Fita adesiva de alumínio 50 mm</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>60 cm</t>
+          <t>1 rolo</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>Canaleta de acrílico ou perfil U de alumínio — leva os cabos do painel à câmara por cima, como na indústria</t>
+          <t>⚠️ Barreira de vapor — obrigatória em todas as juntas do XPS, pelo lado externo (quente)</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr"/>
@@ -2880,21 +2844,21 @@
     </row>
     <row r="91">
       <c r="A91" s="9" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Suportes/mãos-francesas da eletrocalha</t>
+          <t>Manta elastomérica autoadesiva 6 mm</t>
         </is>
       </c>
       <c r="C91" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1 m²</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Cantoneira de alumínio</t>
+          <t>Tipo Armaflex — cantos, arestas e ao redor das passagens de cabo</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr"/>
@@ -2907,21 +2871,21 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>EVA ou MDF 6 mm</t>
+          <t>Espuma expansiva PU (mini)</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
         <is>
-          <t>Bases de máquinas fictícias e plataformas</t>
+          <t>Selagem de passagens de cabo e dreno</t>
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr"/>
@@ -2935,27 +2899,27 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>C.2 — Isolamento térmico</t>
+          <t>C.3 — Vedação, porta e dreno</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>XPS 30 mm (poliestireno extrudado)</t>
+          <t>Perfil EPDM tubular autoadesivo 9 × 6 mm</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>1 m²</t>
+          <t>2 m</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>Isolante principal — k ≈ 0,033 W/m·K. 30 mm, não 20 mm (ver Doc 12)</t>
+          <t>Vedação da porta — perfil tubular comprime muito melhor que o chato de 5 mm</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr"/>
@@ -2968,21 +2932,21 @@
     </row>
     <row r="95">
       <c r="A95" s="9" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>Fita adesiva de alumínio 50 mm</t>
+          <t>Dobradiça piano de alumínio</t>
         </is>
       </c>
       <c r="C95" s="9" t="inlineStr">
         <is>
-          <t>1 rolo</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t>⚠️ Barreira de vapor — obrigatória em todas as juntas do XPS, pelo lado externo (quente)</t>
+          <t>250 mm (cortar de uma barra de 75 cm)</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr"/>
@@ -2995,21 +2959,21 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>Manta elastomérica autoadesiva 6 mm</t>
+          <t>Fecho de pressão (borboleta) inox</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>1 m²</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr">
         <is>
-          <t>Tipo Armaflex — cantos, arestas e ao redor das passagens de cabo</t>
+          <t>Comprime a vedação — tipo fecho de baú</t>
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr"/>
@@ -3022,11 +2986,11 @@
     </row>
     <row r="97">
       <c r="A97" s="9" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>Espuma expansiva PU (mini)</t>
+          <t>Puxador de câmara fria (miniatura)</t>
         </is>
       </c>
       <c r="C97" s="9" t="inlineStr">
@@ -3036,7 +3000,7 @@
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t>Selagem de passagens de cabo e dreno</t>
+          <t>Estética — pode ser um puxador de móvel pequeno</t>
         </is>
       </c>
       <c r="E97" s="10" t="inlineStr"/>
@@ -3047,11 +3011,31 @@
         <v/>
       </c>
     </row>
-    <row r="98" ht="22" customHeight="1">
-      <c r="A98" s="4" t="inlineStr">
-        <is>
-          <t>C.3 — Vedação, porta e dreno</t>
-        </is>
+    <row r="98">
+      <c r="A98" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>Cola S-320 Sinteglas</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>Colagem de acrílico por capilaridade</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr"/>
+      <c r="F98" s="7" t="inlineStr"/>
+      <c r="G98" s="8" t="inlineStr"/>
+      <c r="H98" s="8">
+        <f>IF(C98*G98=0,"",C98*G98)</f>
+        <v/>
       </c>
     </row>
     <row r="99">
@@ -3060,17 +3044,17 @@
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>Perfil EPDM tubular autoadesivo 9 × 6 mm</t>
+          <t>Silicone neutro transparente</t>
         </is>
       </c>
       <c r="C99" s="9" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>1 tubo</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t>Vedação da porta — perfil tubular comprime muito melhor que o chato de 5 mm</t>
+          <t>Vedação de juntas (⚠️ neutro, o acético ataca o acrílico)</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr"/>
@@ -3087,7 +3071,7 @@
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>Dobradiça piano de alumínio</t>
+          <t>Bandeja de alumínio</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
@@ -3097,7 +3081,7 @@
       </c>
       <c r="D100" s="6" t="inlineStr">
         <is>
-          <t>250 mm (cortar de uma barra de 75 cm)</t>
+          <t>~190 × 90 mm — coleta de condensado</t>
         </is>
       </c>
       <c r="E100" s="6" t="inlineStr"/>
@@ -3114,17 +3098,17 @@
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t>Fecho de pressão (borboleta) inox</t>
+          <t>Tubo de silicone Ø 6 mm</t>
         </is>
       </c>
       <c r="C101" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>40 cm</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t>Comprime a vedação — tipo fecho de baú</t>
+          <t>Dreno até o recipiente externo</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr"/>
@@ -3141,17 +3125,17 @@
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>Puxador de câmara fria (miniatura)</t>
+          <t>Sílica gel indicadora</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3 sachês</t>
         </is>
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>Estética — pode ser um puxador de móvel pequeno</t>
+          <t>2 na câmara + 1 dentro da câmara de ar da porta dupla</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr"/>
@@ -3168,17 +3152,17 @@
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>Cola S-320 Sinteglas</t>
+          <t>Recipiente coletor de condensado</t>
         </is>
       </c>
       <c r="C103" s="9" t="inlineStr">
         <is>
-          <t>250 ml</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>Colagem de acrílico por capilaridade</t>
+          <t>Frasco pequeno, embutido na maquete</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr"/>
@@ -3189,40 +3173,20 @@
         <v/>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="B104" s="6" t="inlineStr">
-        <is>
-          <t>Silicone neutro transparente</t>
-        </is>
-      </c>
-      <c r="C104" s="5" t="inlineStr">
-        <is>
-          <t>1 tubo</t>
-        </is>
-      </c>
-      <c r="D104" s="6" t="inlineStr">
-        <is>
-          <t>Vedação de juntas (⚠️ neutro, o acético ataca o acrílico)</t>
-        </is>
-      </c>
-      <c r="E104" s="6" t="inlineStr"/>
-      <c r="F104" s="7" t="inlineStr"/>
-      <c r="G104" s="8" t="inlineStr"/>
-      <c r="H104" s="8">
-        <f>IF(C104*G104=0,"",C104*G104)</f>
-        <v/>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>⚡ CAMADA 2 — PAINEL DE COMANDO</t>
+        </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="9" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t>Bandeja de alumínio</t>
+          <t>Caixa de comando ou MDF</t>
         </is>
       </c>
       <c r="C105" s="9" t="inlineStr">
@@ -3232,7 +3196,7 @@
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t>~190 × 90 mm — coleta de condensado</t>
+          <t>400 × 500 × 200 mm — comprada pronta ou feita em MDF 15 mm</t>
         </is>
       </c>
       <c r="E105" s="10" t="inlineStr"/>
@@ -3245,21 +3209,21 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>Tubo de silicone Ø 6 mm</t>
+          <t>Porta do painel</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>40 cm</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D106" s="6" t="inlineStr">
         <is>
-          <t>Dreno até o recipiente externo</t>
+          <t>MDF 12 mm ou acrílico fumê 5 mm (fica bonito ver os LEDs)</t>
         </is>
       </c>
       <c r="E106" s="6" t="inlineStr"/>
@@ -3272,21 +3236,21 @@
     </row>
     <row r="107">
       <c r="A107" s="9" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t>Sílica gel indicadora</t>
+          <t>Trilho DIN 35 mm</t>
         </is>
       </c>
       <c r="C107" s="9" t="inlineStr">
         <is>
-          <t>3 sachês</t>
+          <t>1,5 m</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t>2 na câmara + 1 dentro da câmara de ar da porta dupla</t>
+          <t>Aço galvanizado — 3 trilhos de ~360 mm</t>
         </is>
       </c>
       <c r="E107" s="10" t="inlineStr"/>
@@ -3299,21 +3263,21 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>Recipiente coletor de condensado</t>
+          <t>Canaleta perfurada 30 × 30 mm</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2 m</t>
         </is>
       </c>
       <c r="D108" s="6" t="inlineStr">
         <is>
-          <t>Frasco pequeno, embutido na maquete</t>
+          <t>Com tampa — organização profissional dos cabos</t>
         </is>
       </c>
       <c r="E108" s="6" t="inlineStr"/>
@@ -3324,11 +3288,31 @@
         <v/>
       </c>
     </row>
-    <row r="109" ht="22" customHeight="1">
-      <c r="A109" s="4" t="inlineStr">
-        <is>
-          <t>⚡ CAMADA 2 — PAINEL DE COMANDO</t>
-        </is>
+    <row r="109">
+      <c r="A109" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="B109" s="10" t="inlineStr">
+        <is>
+          <t>Bloco de distribuição DIN — 1 entrada 4 mm² + 4 saídas</t>
+        </is>
+      </c>
+      <c r="C109" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="inlineStr">
+        <is>
+          <t>BD-POT — 24 V de potência comutados pelo KA2 → BTS #1, BTS #2 e reservas. ⚠️ Cai com a emergência</t>
+        </is>
+      </c>
+      <c r="E109" s="10" t="inlineStr"/>
+      <c r="F109" s="11" t="inlineStr"/>
+      <c r="G109" s="12" t="inlineStr"/>
+      <c r="H109" s="12">
+        <f>IF(C109*G109=0,"",C109*G109)</f>
+        <v/>
       </c>
     </row>
     <row r="110">
@@ -3337,17 +3321,17 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Caixa de comando ou MDF</t>
+          <t>Bloco de distribuição DIN — 1 entrada 2,5 mm² + 4 saídas</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
         <is>
-          <t>400 × 500 × 200 mm — comprada pronta ou feita em MDF 15 mm</t>
+          <t>BD-AUX (12 V auxiliar, do T3) e BD-24V (24 V permanentes: DNLCB30/ESP32, cadeia de comando e o positivo comum dos 4 sinaleiros). ⚠️ Não confundir com o BD-POT — este não cai com a emergência, é o que mantém a supervisão viva para publicar o evento por MQTT</t>
         </is>
       </c>
       <c r="E110" s="6" t="inlineStr"/>
@@ -3364,7 +3348,7 @@
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t>Porta do painel</t>
+          <t>Bloco de distribuição DIN — 1 entrada 2,5 mm² + 6 saídas</t>
         </is>
       </c>
       <c r="C111" s="9" t="inlineStr">
@@ -3374,7 +3358,7 @@
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t>MDF 12 mm ou acrílico fumê 5 mm (fica bonito ver os LEDs)</t>
+          <t>BD-5V — Arduino, Nextion, SD/RTC, lógica dos 2 BTS, LEDs</t>
         </is>
       </c>
       <c r="E111" s="10" t="inlineStr"/>
@@ -3391,17 +3375,17 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>Trilho DIN 35 mm</t>
+          <t>Bloco de distribuição DIN — 1 entrada 10 mm² + 8 saídas</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>1,5 m</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>Aço galvanizado — 3 trilhos de ~360 mm</t>
+          <t>BD-0V — ⭐ o star ground do projeto. Todos os retornos convergem aqui</t>
         </is>
       </c>
       <c r="E112" s="6" t="inlineStr"/>
@@ -3418,17 +3402,17 @@
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t>Canaleta perfurada 30 × 30 mm</t>
+          <t>Bornes DIN parafuso 2,5 mm²</t>
         </is>
       </c>
       <c r="C113" s="9" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t>Com tampa — organização profissional dos cabos</t>
+          <t>Passagem e reservas</t>
         </is>
       </c>
       <c r="E113" s="10" t="inlineStr"/>
@@ -3445,17 +3429,17 @@
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>Bloco de distribuição DIN — 1 entrada 4 mm² + 4 saídas</t>
+          <t>Separadores/tampas de borne</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>BD-POT — 12 V de potência → BTS #1, BTS #2 e reservas</t>
+          <t>Acabamento das réguas</t>
         </is>
       </c>
       <c r="E114" s="6" t="inlineStr"/>
@@ -3472,17 +3456,17 @@
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t>Bloco de distribuição DIN — 1 entrada 2,5 mm² + 4 saídas</t>
+          <t>Alternativa mais barata: bornes comuns + ponte de interligação (pente)</t>
         </is>
       </c>
       <c r="C115" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t>BD-AUX (12 V auxiliar) e BD-24V (24 V)</t>
+          <t>Funciona igual aos blocos, custa menos, menos prático para alterar depois</t>
         </is>
       </c>
       <c r="E115" s="10" t="inlineStr"/>
@@ -3499,17 +3483,17 @@
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>Bloco de distribuição DIN — 1 entrada 2,5 mm² + 6 saídas</t>
+          <t>Identificadores de borne e de cabo</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1 kit</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>BD-5V — Arduino, Nextion, SD/RTC, lógica dos 2 BTS, LEDs</t>
+          <t>Anilhas numeradas — exigido em painel industrial</t>
         </is>
       </c>
       <c r="E116" s="6" t="inlineStr"/>
@@ -3526,17 +3510,17 @@
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t>Bloco de distribuição DIN — 1 entrada 10 mm² + 8 saídas</t>
+          <t>Trava-fim de trilho DIN</t>
         </is>
       </c>
       <c r="C117" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t>BD-0V — ⭐ o star ground do projeto. Todos os retornos convergem aqui</t>
+          <t>Impede os componentes de deslizarem</t>
         </is>
       </c>
       <c r="E117" s="10" t="inlineStr"/>
@@ -3553,17 +3537,17 @@
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>Bornes DIN parafuso 2,5 mm²</t>
+          <t>Botão de Emergência cogumelo 22 mm</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>Passagem e reservas</t>
+          <t>Com trava (girar p/ destravar) — 2 blocos NF (1 para o comando 24 V, 1 para a leitura do Arduino)</t>
         </is>
       </c>
       <c r="E118" s="6" t="inlineStr"/>
@@ -3580,17 +3564,17 @@
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t>Separadores/tampas de borne</t>
+          <t>Botão START 22 mm</t>
         </is>
       </c>
       <c r="C119" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t>Acabamento das réguas</t>
+          <t>Verde, momentâneo — 1 bloco NA (só informa o Arduino)</t>
         </is>
       </c>
       <c r="E119" s="10" t="inlineStr"/>
@@ -3607,17 +3591,17 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>Alternativa mais barata: bornes comuns + ponte de interligação (pente)</t>
+          <t>Botão STOP 22 mm</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>Funciona igual aos blocos, custa menos, menos prático para alterar depois</t>
+          <t>Vermelho, momentâneo — 1 NF (corta o KA2 em 24 V) + 1 NA (avisa o Arduino)</t>
         </is>
       </c>
       <c r="E120" s="6" t="inlineStr"/>
@@ -3634,17 +3618,17 @@
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t>Identificadores de borne e de cabo</t>
+          <t>Botão REARME 22 mm</t>
         </is>
       </c>
       <c r="C121" s="9" t="inlineStr">
         <is>
-          <t>1 kit</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t>Anilhas numeradas — exigido em painel industrial</t>
+          <t>AZUL, momentâneo — 1 bloco NA. Refaz o selo do KA1 após a emergência. Buscar botão pulsador azul 22mm</t>
         </is>
       </c>
       <c r="E121" s="10" t="inlineStr"/>
@@ -3661,17 +3645,17 @@
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>Trava-fim de trilho DIN</t>
+          <t>Blocos de contato 22 mm avulsos</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D122" s="6" t="inlineStr">
         <is>
-          <t>Impede os componentes de deslizarem</t>
+          <t>3 NF + 1 NA: emergência (2 NF), STOP (1 NF + 1 NA). Ver Doc 31 §31.3</t>
         </is>
       </c>
       <c r="E122" s="6" t="inlineStr"/>
@@ -3688,7 +3672,7 @@
       </c>
       <c r="B123" s="10" t="inlineStr">
         <is>
-          <t>Botão de Emergência cogumelo 22 mm</t>
+          <t>Chave seccionadora 24 V no painel</t>
         </is>
       </c>
       <c r="C123" s="9" t="inlineStr">
@@ -3698,7 +3682,7 @@
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t>Com trava (girar p/ destravar) — 2 blocos NF (1 para o comando 24 V, 1 para a leitura do Arduino)</t>
+          <t>Rotativa 2 posições 22 mm — chave geral local da máquina</t>
         </is>
       </c>
       <c r="E123" s="10" t="inlineStr"/>
@@ -3715,17 +3699,17 @@
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>Botão START 22 mm</t>
+          <t>Sinaleiros LED 22 mm 24 V</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>Verde, momentâneo — 1 bloco NA (só informa o Arduino)</t>
+          <t>Verde (RUN), Azul (COOL), Amarelo (HEAT), Vermelho (FAULT). ⚠️ 24 V confirmado — acionados pelo ULN2803 da placa PI-1, alimentados pelo BD-24V permanente (o vermelho de FALHA precisa continuar aceso com a emergência acionada). ~20 mA cada, resistor interno já incluso</t>
         </is>
       </c>
       <c r="E124" s="6" t="inlineStr"/>
@@ -3742,17 +3726,17 @@
       </c>
       <c r="B125" s="10" t="inlineStr">
         <is>
-          <t>Botão STOP 22 mm</t>
+          <t>Prensa-cabo PG9</t>
         </is>
       </c>
       <c r="C125" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t>Vermelho, momentâneo — 1 NF (corta o KA2 em 24 V) + 1 NA (avisa o Arduino)</t>
+          <t>Entrada 24 V de potência (vindo do P1) · saída de potência para a câmara · saída de sinais</t>
         </is>
       </c>
       <c r="E125" s="10" t="inlineStr"/>
@@ -3769,17 +3753,17 @@
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>Botão REARME 22 mm</t>
+          <t>Prensa-cabo PG7</t>
         </is>
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D126" s="6" t="inlineStr">
         <is>
-          <t>AZUL, momentâneo — 1 bloco NA. Refaz o selo do KA1 após a emergência. Buscar botão pulsador azul 22mm</t>
+          <t>Entrada 5 V (do T2) e entrada 12 V auxiliar + 24 V (do T3)</t>
         </is>
       </c>
       <c r="E126" s="6" t="inlineStr"/>
@@ -3796,17 +3780,17 @@
       </c>
       <c r="B127" s="10" t="inlineStr">
         <is>
-          <t>Blocos de contato 22 mm avulsos</t>
+          <t>Bolsa porta-documentos p/ porta</t>
         </is>
       </c>
       <c r="C127" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t>3 NF + 1 NA: emergência (2 NF), STOP (1 NF + 1 NA). Ver Doc 31 §31.3</t>
+          <t>Guarda o diagrama elétrico — padrão em painel industrial</t>
         </is>
       </c>
       <c r="E127" s="10" t="inlineStr"/>
@@ -3817,50 +3801,30 @@
         <v/>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="5" t="n">
-        <v>113</v>
-      </c>
-      <c r="B128" s="6" t="inlineStr">
-        <is>
-          <t>Chave seccionadora 24 V no painel</t>
-        </is>
-      </c>
-      <c r="C128" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D128" s="6" t="inlineStr">
-        <is>
-          <t>Rotativa 2 posições 22 mm — chave geral local da máquina</t>
-        </is>
-      </c>
-      <c r="E128" s="6" t="inlineStr"/>
-      <c r="F128" s="7" t="inlineStr"/>
-      <c r="G128" s="8" t="inlineStr"/>
-      <c r="H128" s="8">
-        <f>IF(C128*G128=0,"",C128*G128)</f>
-        <v/>
+    <row r="128" ht="22" customHeight="1">
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>L.1 — Controle e interface</t>
+        </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="9" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B129" s="10" t="inlineStr">
         <is>
-          <t>Sinaleiros LED 22 mm 24 V</t>
+          <t>Arduino Mega 2560 R3</t>
         </is>
       </c>
       <c r="C129" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t>Verde (RUN), Azul (COOL), Amarelo (HEAT), Vermelho (FAULT)</t>
+          <t>ATmega2560, 54 GPIO, 4 UARTs</t>
         </is>
       </c>
       <c r="E129" s="10" t="inlineStr"/>
@@ -3873,21 +3837,21 @@
     </row>
     <row r="130">
       <c r="A130" s="5" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>Prensa-cabo PG9</t>
+          <t>Shield de expansão Mega (bornes parafuso)</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D130" s="6" t="inlineStr">
         <is>
-          <t>Entrada 12 V potência · saída de potência · saída de sinais</t>
+          <t>Sensor Shield V2.0</t>
         </is>
       </c>
       <c r="E130" s="6" t="inlineStr"/>
@@ -3900,21 +3864,21 @@
     </row>
     <row r="131">
       <c r="A131" s="9" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t>Prensa-cabo PG7</t>
+          <t>Suporte DIN para Arduino Mega</t>
         </is>
       </c>
       <c r="C131" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t>Entrada 5 V (do T2) e entrada 12 V auxiliar + 24 V (do T3)</t>
+          <t>Ou SPCI4/adaptador</t>
         </is>
       </c>
       <c r="E131" s="10" t="inlineStr"/>
@@ -3927,11 +3891,11 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>Bolsa porta-documentos p/ porta</t>
+          <t>Tela Nextion Basic 3.2"</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
@@ -3941,7 +3905,7 @@
       </c>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t>Guarda o diagrama elétrico — padrão em painel industrial</t>
+          <t>NX4024T032, 400×240, TTL 5 V</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr"/>
@@ -3952,11 +3916,31 @@
         <v/>
       </c>
     </row>
-    <row r="133" ht="22" customHeight="1">
-      <c r="A133" s="4" t="inlineStr">
-        <is>
-          <t>L.1 — Controle e interface</t>
-        </is>
+    <row r="133">
+      <c r="A133" s="9" t="n">
+        <v>117</v>
+      </c>
+      <c r="B133" s="10" t="inlineStr">
+        <is>
+          <t>ESP32-WROOM-32U</t>
+        </is>
+      </c>
+      <c r="C133" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D133" s="10" t="inlineStr">
+        <is>
+          <t>30 pinos, conector de antena IPEX</t>
+        </is>
+      </c>
+      <c r="E133" s="10" t="inlineStr"/>
+      <c r="F133" s="11" t="inlineStr"/>
+      <c r="G133" s="12" t="inlineStr"/>
+      <c r="H133" s="12">
+        <f>IF(C133*G133=0,"",C133*G133)</f>
+        <v/>
       </c>
     </row>
     <row r="134">
@@ -3965,7 +3949,7 @@
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>Arduino Mega 2560 R3</t>
+          <t>DNLCB30 — base DIN para ESP32</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
@@ -3975,7 +3959,7 @@
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>ATmega2560, 54 GPIO, 4 UARTs</t>
+          <t>Entrada 7–35 V (alimentada direto do barramento 24 V), conversão 3,3 ↔ 5 V automática. Não inclui o ESP32</t>
         </is>
       </c>
       <c r="E134" s="6" t="inlineStr"/>
@@ -3992,7 +3976,7 @@
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t>Shield de expansão Mega (bornes parafuso)</t>
+          <t>Pigtail IPEX (u.FL) → SMA macho, 20–30 cm</t>
         </is>
       </c>
       <c r="C135" s="9" t="inlineStr">
@@ -4002,7 +3986,7 @@
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t>Sensor Shield V2.0</t>
+          <t>Liga o ESP32 ao conector de painel</t>
         </is>
       </c>
       <c r="E135" s="10" t="inlineStr"/>
@@ -4019,7 +4003,7 @@
       </c>
       <c r="B136" s="6" t="inlineStr">
         <is>
-          <t>Suporte DIN para Arduino Mega</t>
+          <t>Conector SMA fêmea de painel (bulkhead)</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
@@ -4029,7 +4013,7 @@
       </c>
       <c r="D136" s="6" t="inlineStr">
         <is>
-          <t>Ou SPCI4/adaptador</t>
+          <t>Rosca de painel Ø 6,5 mm, com porca e arruela de pressão. ⚠️ Nunca passar o coaxial por prensa-cabo</t>
         </is>
       </c>
       <c r="E136" s="6" t="inlineStr"/>
@@ -4046,7 +4030,7 @@
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>Tela Nextion Basic 3.2"</t>
+          <t>Antena 2,4 GHz SMA macho 3 dBi articulável</t>
         </is>
       </c>
       <c r="C137" s="9" t="inlineStr">
@@ -4056,7 +4040,7 @@
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t>NX4024T032, 400×240, TTL 5 V</t>
+          <t>Rosqueada por fora, na lateral direita, parte alta do painel</t>
         </is>
       </c>
       <c r="E137" s="10" t="inlineStr"/>
@@ -4073,7 +4057,7 @@
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
-          <t>ESP32-WROOM-32U</t>
+          <t>Módulo Micro SD (SPI)</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
@@ -4083,7 +4067,7 @@
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>30 pinos, conector de antena IPEX</t>
+          <t>5 V, com regulador e level shifter</t>
         </is>
       </c>
       <c r="E138" s="6" t="inlineStr"/>
@@ -4100,7 +4084,7 @@
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t>DNLCB30 — base DIN para ESP32</t>
+          <t>Cartão Micro SD</t>
         </is>
       </c>
       <c r="C139" s="9" t="inlineStr">
@@ -4110,7 +4094,7 @@
       </c>
       <c r="D139" s="10" t="inlineStr">
         <is>
-          <t>Entrada 7–35 V (alimentada direto do barramento 24 V), conversão 3,3 ↔ 5 V automática. Não inclui o ESP32</t>
+          <t>8–16 GB, Classe 10</t>
         </is>
       </c>
       <c r="E139" s="10" t="inlineStr"/>
@@ -4127,7 +4111,7 @@
       </c>
       <c r="B140" s="6" t="inlineStr">
         <is>
-          <t>Pigtail IPEX (u.FL) → SMA macho, 20–30 cm</t>
+          <t>Módulo RTC DS3231</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
@@ -4137,7 +4121,7 @@
       </c>
       <c r="D140" s="6" t="inlineStr">
         <is>
-          <t>Liga o ESP32 ao conector de painel</t>
+          <t>I²C, ±2 ppm</t>
         </is>
       </c>
       <c r="E140" s="6" t="inlineStr"/>
@@ -4154,7 +4138,7 @@
       </c>
       <c r="B141" s="10" t="inlineStr">
         <is>
-          <t>Conector SMA fêmea de painel (bulkhead)</t>
+          <t>Bateria CR2032</t>
         </is>
       </c>
       <c r="C141" s="9" t="inlineStr">
@@ -4164,7 +4148,7 @@
       </c>
       <c r="D141" s="10" t="inlineStr">
         <is>
-          <t>Rosca de painel Ø 6,5 mm, com porca e arruela de pressão. ⚠️ Nunca passar o coaxial por prensa-cabo</t>
+          <t>Backup do RTC</t>
         </is>
       </c>
       <c r="E141" s="10" t="inlineStr"/>
@@ -4175,50 +4159,30 @@
         <v/>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="5" t="n">
-        <v>126</v>
-      </c>
-      <c r="B142" s="6" t="inlineStr">
-        <is>
-          <t>Antena 2,4 GHz SMA macho 3 dBi articulável</t>
-        </is>
-      </c>
-      <c r="C142" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D142" s="6" t="inlineStr">
-        <is>
-          <t>Rosqueada por fora, na lateral direita, parte alta do painel</t>
-        </is>
-      </c>
-      <c r="E142" s="6" t="inlineStr"/>
-      <c r="F142" s="7" t="inlineStr"/>
-      <c r="G142" s="8" t="inlineStr"/>
-      <c r="H142" s="8">
-        <f>IF(C142*G142=0,"",C142*G142)</f>
-        <v/>
+    <row r="142" ht="22" customHeight="1">
+      <c r="A142" s="4" t="inlineStr">
+        <is>
+          <t>L.2 — Potência e acionamento</t>
+        </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="9" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B143" s="10" t="inlineStr">
         <is>
-          <t>Módulo Micro SD (SPI)</t>
+          <t>Driver ponte-H BTS7960</t>
         </is>
       </c>
       <c r="C143" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D143" s="10" t="inlineStr">
         <is>
-          <t>5 V, com regulador e level shifter</t>
+          <t>43 A, pino IS de diagnóstico</t>
         </is>
       </c>
       <c r="E143" s="10" t="inlineStr"/>
@@ -4231,21 +4195,21 @@
     </row>
     <row r="144">
       <c r="A144" s="5" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B144" s="6" t="inlineStr">
         <is>
-          <t>Cartão Micro SD</t>
+          <t>Suporte SPCI4 trilho DIN</t>
         </is>
       </c>
       <c r="C144" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D144" s="6" t="inlineStr">
         <is>
-          <t>8–16 GB, Classe 10</t>
+          <t>Fixa PCI 100 × 79 mm</t>
         </is>
       </c>
       <c r="E144" s="6" t="inlineStr"/>
@@ -4258,11 +4222,11 @@
     </row>
     <row r="145">
       <c r="A145" s="9" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B145" s="10" t="inlineStr">
         <is>
-          <t>Módulo RTC DS3231</t>
+          <t>Cooler 40 mm 12 V</t>
         </is>
       </c>
       <c r="C145" s="9" t="inlineStr">
@@ -4272,7 +4236,7 @@
       </c>
       <c r="D145" s="10" t="inlineStr">
         <is>
-          <t>I²C, ±2 ppm</t>
+          <t>Refrigeração dos BTS</t>
         </is>
       </c>
       <c r="E145" s="10" t="inlineStr"/>
@@ -4285,11 +4249,11 @@
     </row>
     <row r="146">
       <c r="A146" s="5" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B146" s="6" t="inlineStr">
         <is>
-          <t>Bateria CR2032</t>
+          <t>KA1 — Relé de interface 24 Vcc, 2 contatos</t>
         </is>
       </c>
       <c r="C146" s="5" t="inlineStr">
@@ -4299,7 +4263,7 @@
       </c>
       <c r="D146" s="6" t="inlineStr">
         <is>
-          <t>Backup do RTC</t>
+          <t>Faz o selo (habilitação) e alimenta a bobina do KA2. Conduz só miliampères — 6 A basta. Buscar relé de interface 24vdc 2 contatos din. Premium: Finder 55.32.9.024.0040</t>
         </is>
       </c>
       <c r="E146" s="6" t="inlineStr"/>
@@ -4310,11 +4274,31 @@
         <v/>
       </c>
     </row>
-    <row r="147" ht="22" customHeight="1">
-      <c r="A147" s="4" t="inlineStr">
-        <is>
-          <t>L.2 — Potência e acionamento</t>
-        </is>
+    <row r="147">
+      <c r="A147" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="B147" s="10" t="inlineStr">
+        <is>
+          <t>KA2 — Relé de interface 24 Vcc, contato ≥ 10 A</t>
+        </is>
+      </c>
+      <c r="C147" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D147" s="10" t="inlineStr">
+        <is>
+          <t>É ele que chaveia os 24 V / 6,0 A de potência dos BTS. ⚠️ Confirme os 10 A no anúncio — a maioria dos slim é de 6 A — e confirme que a corrente é declarada em DC: muito relé de 10 A/250 VAC cai para 5 A ou menos em 24 Vcc, porque corrente contínua não tem passagem por zero e o arco custa mais a extinguir. Buscar relé de interface 24vdc 10a trilho din. Premium: Finder 46.61.9.024.0040 + base 95.05 (16 A)</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr"/>
+      <c r="F147" s="11" t="inlineStr"/>
+      <c r="G147" s="12" t="inlineStr"/>
+      <c r="H147" s="12">
+        <f>IF(C147*G147=0,"",C147*G147)</f>
+        <v/>
       </c>
     </row>
     <row r="148">
@@ -4323,17 +4307,17 @@
       </c>
       <c r="B148" s="6" t="inlineStr">
         <is>
-          <t>Driver ponte-H BTS7960</t>
+          <t>Resistor 10 kΩ 1/4 W</t>
         </is>
       </c>
       <c r="C148" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D148" s="6" t="inlineStr">
         <is>
-          <t>43 A, pino IS de diagnóstico</t>
+          <t>Pull-down em cada R_EN dos BTS7960 (2) + reservas. ⚠️ Garante que pino solto = driver desligado — ficou ainda mais crítico com os 24 V permanentes na entrada dos BTS</t>
         </is>
       </c>
       <c r="E148" s="6" t="inlineStr"/>
@@ -4350,7 +4334,7 @@
       </c>
       <c r="B149" s="10" t="inlineStr">
         <is>
-          <t>Suporte SPCI4 trilho DIN</t>
+          <t>Resistor 22 kΩ 1/4 W ⬆</t>
         </is>
       </c>
       <c r="C149" s="9" t="inlineStr">
@@ -4360,7 +4344,7 @@
       </c>
       <c r="D149" s="10" t="inlineStr">
         <is>
-          <t>Fixa PCI 100 × 79 mm</t>
+          <t>Braço superior do divisor de realimentação de tensão para o pino D25</t>
         </is>
       </c>
       <c r="E149" s="10" t="inlineStr"/>
@@ -4377,17 +4361,17 @@
       </c>
       <c r="B150" s="6" t="inlineStr">
         <is>
-          <t>Cooler 40 mm 12 V</t>
+          <t>Resistor 4,7 kΩ 1/4 W</t>
         </is>
       </c>
       <c r="C150" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D150" s="6" t="inlineStr">
         <is>
-          <t>Refrigeração dos BTS</t>
+          <t>Braço inferior do mesmo divisor</t>
         </is>
       </c>
       <c r="E150" s="6" t="inlineStr"/>
@@ -4398,50 +4382,30 @@
         <v/>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="9" t="n">
-        <v>134</v>
-      </c>
-      <c r="B151" s="10" t="inlineStr">
-        <is>
-          <t>KA1 — Relé de interface 24 Vcc, 2 contatos</t>
-        </is>
-      </c>
-      <c r="C151" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D151" s="10" t="inlineStr">
-        <is>
-          <t>Faz o selo (habilitação) e alimenta a bobina do KA2. Conduz só miliampères — 6 A basta. Buscar relé de interface 24vdc 2 contatos din. Premium: Finder 55.32.9.024.0040</t>
-        </is>
-      </c>
-      <c r="E151" s="10" t="inlineStr"/>
-      <c r="F151" s="11" t="inlineStr"/>
-      <c r="G151" s="12" t="inlineStr"/>
-      <c r="H151" s="12">
-        <f>IF(C151*G151=0,"",C151*G151)</f>
-        <v/>
+    <row r="151" ht="22" customHeight="1">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>L.3 — Atuadores térmicos e ventilação</t>
+        </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="5" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B152" s="6" t="inlineStr">
         <is>
-          <t>KA2 — Relé de interface 24 Vcc, contato ≥ 10 A</t>
+          <t>Pastilha Peltier TEC1-12706</t>
         </is>
       </c>
       <c r="C152" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D152" s="6" t="inlineStr">
         <is>
-          <t>É ele que chaveia os 12 V / 6,3 A dos BTS. ⚠️ Confirme os 10 A no anúncio — a maioria dos slim é de 6 A. Buscar relé de interface 24vdc 10a trilho din. Premium: Finder 46.61.9.024.0040 + base 95.05 (16 A)</t>
+          <t>12 V / ~6 A / 60 W cada. 2 em uso, ligadas EM SÉRIE (24 V / 6,0 A / 144 W) + 1 reserva. ⚠️ Comprar do mesmo lote/vendedor — em série as duas conduzem a mesma corrente, e pastilhas descasadas trabalham desequilibradas</t>
         </is>
       </c>
       <c r="E152" s="6" t="inlineStr"/>
@@ -4454,21 +4418,21 @@
     </row>
     <row r="153">
       <c r="A153" s="9" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B153" s="10" t="inlineStr">
         <is>
-          <t>Resistor 10 kΩ 1/4 W</t>
+          <t>Aquecedor PTC cerâmico 24 V / 60 W</t>
         </is>
       </c>
       <c r="C153" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D153" s="10" t="inlineStr">
         <is>
-          <t>Pull-down em cada R_EN dos BTS7960 (2) + divisor de realimentação (1) + reserva. ⚠️ Garante que pino solto = driver desligado</t>
+          <t>Com aletas, versão de 24 V (2,5 A) para ligar direto no barramento. 60 W, não 100 W — equilibra as duas potências. ⚠️ Menos comum que o de 12 V: comprar cedo, no Lote A. Buscar também como aquecedor ar quente ptc 24v (incubadora / impressora 3D)</t>
         </is>
       </c>
       <c r="E153" s="10" t="inlineStr"/>
@@ -4481,11 +4445,11 @@
     </row>
     <row r="154">
       <c r="A154" s="5" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B154" s="6" t="inlineStr">
         <is>
-          <t>Resistor 4,7 kΩ 1/4 W</t>
+          <t>Dissipador + cooler 80 mm p/ lado quente da Peltier</t>
         </is>
       </c>
       <c r="C154" s="5" t="inlineStr">
@@ -4495,7 +4459,7 @@
       </c>
       <c r="D154" s="6" t="inlineStr">
         <is>
-          <t>Divisor de realimentação do 12 V para o pino D25</t>
+          <t>Um para cada pastilha. ⚠️ 3 fios (com sinal de RPM) nos dois — o firmware monitora os dois tacômetros e bloqueia a refrigeração se qualquer um parar</t>
         </is>
       </c>
       <c r="E154" s="6" t="inlineStr"/>
@@ -4508,21 +4472,21 @@
     </row>
     <row r="155">
       <c r="A155" s="9" t="n">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B155" s="10" t="inlineStr">
         <is>
-          <t>Diodo 1N4007</t>
+          <t>Pasta térmica</t>
         </is>
       </c>
       <c r="C155" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D155" s="10" t="inlineStr">
         <is>
-          <t>Proteção geral e reservas (o relé de interface já traz o roda-livre interno)</t>
+          <t>Seringa 5 g — dá para os 2 conjuntos</t>
         </is>
       </c>
       <c r="E155" s="10" t="inlineStr"/>
@@ -4533,11 +4497,31 @@
         <v/>
       </c>
     </row>
-    <row r="156" ht="22" customHeight="1">
-      <c r="A156" s="4" t="inlineStr">
-        <is>
-          <t>L.3 — Atuadores térmicos e ventilação</t>
-        </is>
+    <row r="156">
+      <c r="A156" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="B156" s="6" t="inlineStr">
+        <is>
+          <t>Fan 60 × 60 mm 12 V</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D156" s="6" t="inlineStr">
+        <is>
+          <t>Internas — lado PTC (1 sopra ↑, 1 sopra ↓)</t>
+        </is>
+      </c>
+      <c r="E156" s="6" t="inlineStr"/>
+      <c r="F156" s="7" t="inlineStr"/>
+      <c r="G156" s="8" t="inlineStr"/>
+      <c r="H156" s="8">
+        <f>IF(C156*G156=0,"",C156*G156)</f>
+        <v/>
       </c>
     </row>
     <row r="157">
@@ -4546,17 +4530,17 @@
       </c>
       <c r="B157" s="10" t="inlineStr">
         <is>
-          <t>Pastilha Peltier TEC1-12706</t>
+          <t>Fan 40 × 40 mm 12 V</t>
         </is>
       </c>
       <c r="C157" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D157" s="10" t="inlineStr">
         <is>
-          <t>12 V, ~6 A, 60 W (+1 reserva é sábio)</t>
+          <t>Internas — lado Peltier (1 sopra ↓, 1 sopra ↑)</t>
         </is>
       </c>
       <c r="E157" s="10" t="inlineStr"/>
@@ -4567,40 +4551,20 @@
         <v/>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" s="5" t="n">
-        <v>140</v>
-      </c>
-      <c r="B158" s="6" t="inlineStr">
-        <is>
-          <t>Aquecedor PTC cerâmico 12 V 60 W</t>
-        </is>
-      </c>
-      <c r="C158" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D158" s="6" t="inlineStr">
-        <is>
-          <t>Com aletas. 60 W, não 100 W — equilibra as duas potências e alivia o T1</t>
-        </is>
-      </c>
-      <c r="E158" s="6" t="inlineStr"/>
-      <c r="F158" s="7" t="inlineStr"/>
-      <c r="G158" s="8" t="inlineStr"/>
-      <c r="H158" s="8">
-        <f>IF(C158*G158=0,"",C158*G158)</f>
-        <v/>
+    <row r="158" ht="22" customHeight="1">
+      <c r="A158" s="4" t="inlineStr">
+        <is>
+          <t>L.4 — Sensores</t>
+        </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="9" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B159" s="10" t="inlineStr">
         <is>
-          <t>Dissipador + cooler 80 mm p/ lado quente da Peltier</t>
+          <t>Sensor DS18B20 à prova d'água</t>
         </is>
       </c>
       <c r="C159" s="9" t="inlineStr">
@@ -4610,7 +4574,7 @@
       </c>
       <c r="D159" s="10" t="inlineStr">
         <is>
-          <t>3 fios (com sinal de RPM) — obrigatório para a proteção</t>
+          <t>1-Wire, ±0,5 °C — centro da câmara</t>
         </is>
       </c>
       <c r="E159" s="10" t="inlineStr"/>
@@ -4623,21 +4587,21 @@
     </row>
     <row r="160">
       <c r="A160" s="5" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B160" s="6" t="inlineStr">
         <is>
-          <t>Pasta térmica</t>
+          <t>Resistor 4,7 kΩ 1/4 W</t>
         </is>
       </c>
       <c r="C160" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D160" s="6" t="inlineStr">
         <is>
-          <t>Seringa 5 g</t>
+          <t>Pull-up do barramento 1-Wire</t>
         </is>
       </c>
       <c r="E160" s="6" t="inlineStr"/>
@@ -4650,21 +4614,21 @@
     </row>
     <row r="161">
       <c r="A161" s="9" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B161" s="10" t="inlineStr">
         <is>
-          <t>Fan 60 × 60 mm 12 V</t>
+          <t>Sensor AM2315C</t>
         </is>
       </c>
       <c r="C161" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D161" s="10" t="inlineStr">
         <is>
-          <t>Internas — lado PTC (1 sopra ↑, 1 sopra ↓)</t>
+          <t>I²C, umidade + temperatura, carcaça selada</t>
         </is>
       </c>
       <c r="E161" s="10" t="inlineStr"/>
@@ -4677,21 +4641,21 @@
     </row>
     <row r="162">
       <c r="A162" s="5" t="n">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B162" s="6" t="inlineStr">
         <is>
-          <t>Fan 40 × 40 mm 12 V</t>
+          <t>Capacitor cerâmico 100 nF</t>
         </is>
       </c>
       <c r="C162" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D162" s="6" t="inlineStr">
         <is>
-          <t>Internas — lado Peltier (1 sopra ↓, 1 sopra ↑)</t>
+          <t>Filtro dos pinos IS dos BTS (2) + filtro do divisor D25 (1) + reservas</t>
         </is>
       </c>
       <c r="E162" s="6" t="inlineStr"/>
@@ -4702,57 +4666,57 @@
         <v/>
       </c>
     </row>
-    <row r="163" ht="22" customHeight="1">
-      <c r="A163" s="4" t="inlineStr">
-        <is>
-          <t>L.4 — Sensores</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="5" t="n">
-        <v>145</v>
-      </c>
-      <c r="B164" s="6" t="inlineStr">
-        <is>
-          <t>Sensor DS18B20 à prova d'água</t>
-        </is>
-      </c>
-      <c r="C164" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D164" s="6" t="inlineStr">
-        <is>
-          <t>1-Wire, ±0,5 °C — centro da câmara</t>
-        </is>
-      </c>
-      <c r="E164" s="6" t="inlineStr"/>
-      <c r="F164" s="7" t="inlineStr"/>
-      <c r="G164" s="8" t="inlineStr"/>
-      <c r="H164" s="8">
-        <f>IF(C164*G164=0,"",C164*G164)</f>
-        <v/>
+    <row r="163">
+      <c r="A163" s="9" t="n">
+        <v>144</v>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>Resistor 220 Ω 1/4 W</t>
+        </is>
+      </c>
+      <c r="C163" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D163" s="10" t="inlineStr">
+        <is>
+          <t>4 usos + 2 reservas — série dos LEDs brancos da iluminação da maquete (5 V). ⚠️ Não são mais dos sinaleiros do painel, que agora são de 24 V</t>
+        </is>
+      </c>
+      <c r="E163" s="10" t="inlineStr"/>
+      <c r="F163" s="11" t="inlineStr"/>
+      <c r="G163" s="12" t="inlineStr"/>
+      <c r="H163" s="12">
+        <f>IF(C163*G163=0,"",C163*G163)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164" ht="22" customHeight="1">
+      <c r="A164" s="4" t="inlineStr">
+        <is>
+          <t>L.5 — Placa de Interface PI-1 (onde os componentes discretos moram)</t>
+        </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="9" t="n">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B165" s="10" t="inlineStr">
         <is>
-          <t>Resistor 4,7 kΩ 1/4 W</t>
+          <t>Placa ilhada (padrão furos isolados)</t>
         </is>
       </c>
       <c r="C165" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D165" s="10" t="inlineStr">
         <is>
-          <t>Pull-up do barramento 1-Wire</t>
+          <t>~5 × 7 cm. ⚠️ Ilhada, não de barramento — na de barramento você acaba tendo que cortar trilha, e é dali que saem os curtos difíceis de achar</t>
         </is>
       </c>
       <c r="E165" s="10" t="inlineStr"/>
@@ -4765,11 +4729,11 @@
     </row>
     <row r="166">
       <c r="A166" s="5" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B166" s="6" t="inlineStr">
         <is>
-          <t>Sensor AM2315C</t>
+          <t>Caixa modular para trilho DIN — 3 módulos (52,5 mm)</t>
         </is>
       </c>
       <c r="C166" s="5" t="inlineStr">
@@ -4779,7 +4743,7 @@
       </c>
       <c r="D166" s="6" t="inlineStr">
         <is>
-          <t>I²C, umidade + temperatura, carcaça selada</t>
+          <t>Invólucro da PI-1. Cabe no espaço livre do trilho 3, ao lado do Arduino. Buscar caixa para trilho din 3m modular</t>
         </is>
       </c>
       <c r="E166" s="6" t="inlineStr"/>
@@ -4792,21 +4756,21 @@
     </row>
     <row r="167">
       <c r="A167" s="9" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B167" s="10" t="inlineStr">
         <is>
-          <t>Capacitor cerâmico 100 nF</t>
+          <t>Borne KF350 / KRE passo 3,5 mm — 10 vias</t>
         </is>
       </c>
       <c r="C167" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D167" s="10" t="inlineStr">
         <is>
-          <t>Filtro dos pinos IS dos BTS</t>
+          <t>Um borne superior (lado Arduino) e um inferior (lado campo). Passo de 3,5 mm porque todos os cabos são de 0,25 mm²</t>
         </is>
       </c>
       <c r="E167" s="10" t="inlineStr"/>
@@ -4819,21 +4783,21 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B168" s="6" t="inlineStr">
         <is>
-          <t>Resistor 220 Ω 1/4 W</t>
+          <t>CI ULN2803A (DIP 18 pinos)</t>
         </is>
       </c>
       <c r="C168" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D168" s="6" t="inlineStr">
         <is>
-          <t>Série dos LEDs de sinalização</t>
+          <t>Driver dos 4 sinaleiros de 24 V — 8 canais Darlington, 500 mA/50 V, com diodos de proteção internos. 1 uso + 1 reserva (o CI é barato e é o único ponto onde 24 V encosta na lógica)</t>
         </is>
       </c>
       <c r="E168" s="6" t="inlineStr"/>
@@ -4844,11 +4808,31 @@
         <v/>
       </c>
     </row>
-    <row r="169" ht="22" customHeight="1">
-      <c r="A169" s="4" t="inlineStr">
-        <is>
-          <t>🔧 CAMADA 3 — CABOS E ACESSÓRIOS</t>
-        </is>
+    <row r="169">
+      <c r="A169" s="9" t="n">
+        <v>149</v>
+      </c>
+      <c r="B169" s="10" t="inlineStr">
+        <is>
+          <t>Soquete DIP 18 pinos</t>
+        </is>
+      </c>
+      <c r="C169" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D169" s="10" t="inlineStr">
+        <is>
+          <t>⚠️ Solde o soquete, não o CI. Permite trocar o chip sem dessoldar nada</t>
+        </is>
+      </c>
+      <c r="E169" s="10" t="inlineStr"/>
+      <c r="F169" s="11" t="inlineStr"/>
+      <c r="G169" s="12" t="inlineStr"/>
+      <c r="H169" s="12">
+        <f>IF(C169*G169=0,"",C169*G169)</f>
+        <v/>
       </c>
     </row>
     <row r="170">
@@ -4857,24 +4841,20 @@
       </c>
       <c r="B170" s="6" t="inlineStr">
         <is>
-          <t>Cabo flexível 1,5 mm² preto</t>
+          <t>Fio rígido 0,25 mm² para interligação</t>
         </is>
       </c>
       <c r="C170" s="5" t="inlineStr">
         <is>
-          <t>3 m</t>
+          <t>1 m</t>
         </is>
       </c>
       <c r="D170" s="6" t="inlineStr">
         <is>
-          <t>750 V</t>
-        </is>
-      </c>
-      <c r="E170" s="6" t="inlineStr">
-        <is>
-          <t>Retorno geral 0 V e 12 V de potência</t>
-        </is>
-      </c>
+          <t>Ligações por baixo da placa. ⚠️ Não usar "sobra de perna" de componente em trecho longo — oxida e não é isolada</t>
+        </is>
+      </c>
+      <c r="E170" s="6" t="inlineStr"/>
       <c r="F170" s="7" t="inlineStr"/>
       <c r="G170" s="8" t="inlineStr"/>
       <c r="H170" s="8">
@@ -4888,24 +4868,20 @@
       </c>
       <c r="B171" s="10" t="inlineStr">
         <is>
-          <t>Cabo flexível 1,5 mm² vermelho</t>
+          <t>Verniz spray para PCI (ou esmalte incolor)</t>
         </is>
       </c>
       <c r="C171" s="9" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D171" s="10" t="inlineStr">
         <is>
-          <t>750 V</t>
-        </is>
-      </c>
-      <c r="E171" s="10" t="inlineStr">
-        <is>
-          <t>12 V de potência (BTS)</t>
-        </is>
-      </c>
+          <t>Proteção do lado da solda contra umidade e oxidação</t>
+        </is>
+      </c>
+      <c r="E171" s="10" t="inlineStr"/>
       <c r="F171" s="11" t="inlineStr"/>
       <c r="G171" s="12" t="inlineStr"/>
       <c r="H171" s="12">
@@ -4919,24 +4895,20 @@
       </c>
       <c r="B172" s="6" t="inlineStr">
         <is>
-          <t>Cabo flexível 0,75 mm² vermelho/preto</t>
+          <t>Termorretrátil Ø 2 mm</t>
         </is>
       </c>
       <c r="C172" s="5" t="inlineStr">
         <is>
-          <t>3 m</t>
+          <t>30 cm</t>
         </is>
       </c>
       <c r="D172" s="6" t="inlineStr">
         <is>
-          <t>750 V</t>
-        </is>
-      </c>
-      <c r="E172" s="6" t="inlineStr">
-        <is>
-          <t>Barramento 24 V (trechos internos)</t>
-        </is>
-      </c>
+          <t>Isolação dos 2 resistores de 10 kΩ soldados nos BTS7960</t>
+        </is>
+      </c>
+      <c r="E172" s="6" t="inlineStr"/>
       <c r="F172" s="7" t="inlineStr"/>
       <c r="G172" s="8" t="inlineStr"/>
       <c r="H172" s="8">
@@ -4950,24 +4922,20 @@
       </c>
       <c r="B173" s="10" t="inlineStr">
         <is>
-          <t>Cabo flexível 0,5 mm² (5 cores)</t>
+          <t>Etiqueta impressa em papel adesivo</t>
         </is>
       </c>
       <c r="C173" s="9" t="inlineStr">
         <is>
-          <t>10 m</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D173" s="10" t="inlineStr">
         <is>
-          <t>750 V</t>
-        </is>
-      </c>
-      <c r="E173" s="10" t="inlineStr">
-        <is>
-          <t>5 V, 12 V auxiliar</t>
-        </is>
-      </c>
+          <t>Identificação das 20 vias na frente da caixa — é o que torna a placa auditável</t>
+        </is>
+      </c>
+      <c r="E173" s="10" t="inlineStr"/>
       <c r="F173" s="11" t="inlineStr"/>
       <c r="G173" s="12" t="inlineStr"/>
       <c r="H173" s="12">
@@ -4975,59 +4943,35 @@
         <v/>
       </c>
     </row>
-    <row r="174">
-      <c r="A174" s="5" t="n">
-        <v>154</v>
-      </c>
-      <c r="B174" s="6" t="inlineStr">
-        <is>
-          <t>Cabo flexível 0,25 mm² (8 cores)</t>
-        </is>
-      </c>
-      <c r="C174" s="5" t="inlineStr">
-        <is>
-          <t>15 m</t>
-        </is>
-      </c>
-      <c r="D174" s="6" t="inlineStr">
-        <is>
-          <t>Sinais</t>
-        </is>
-      </c>
-      <c r="E174" s="6" t="inlineStr">
-        <is>
-          <t>Sensores, botões, comunicação</t>
-        </is>
-      </c>
-      <c r="F174" s="7" t="inlineStr"/>
-      <c r="G174" s="8" t="inlineStr"/>
-      <c r="H174" s="8">
-        <f>IF(C174*G174=0,"",C174*G174)</f>
-        <v/>
+    <row r="174" ht="22" customHeight="1">
+      <c r="A174" s="4" t="inlineStr">
+        <is>
+          <t>🔧 CAMADA 3 — CABOS E ACESSÓRIOS</t>
+        </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="9" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B175" s="10" t="inlineStr">
         <is>
-          <t>Cabo par trançado blindado 2×0,25 mm²</t>
+          <t>Cabo flexível 1,5 mm² preto</t>
         </is>
       </c>
       <c r="C175" s="9" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>3 m</t>
         </is>
       </c>
       <c r="D175" s="10" t="inlineStr">
         <is>
-          <t>Blindado, malha aterrada em um ponto</t>
+          <t>750 V</t>
         </is>
       </c>
       <c r="E175" s="10" t="inlineStr">
         <is>
-          <t>I²C e 1-Wire (trecho câmara → painel)</t>
+          <t>Retorno geral 0 V (6,9 A — soma dos 3 ramais)</t>
         </is>
       </c>
       <c r="F175" s="11" t="inlineStr"/>
@@ -5039,26 +4983,26 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B176" s="6" t="inlineStr">
         <is>
-          <t>Terminal tubular (ilhós) 0,25 / 0,5 / 1,5 mm²</t>
+          <t>Cabo flexível 1,5 mm² vermelho</t>
         </is>
       </c>
       <c r="C176" s="5" t="inlineStr">
         <is>
-          <t>1 kit</t>
+          <t>2 m</t>
         </is>
       </c>
       <c r="D176" s="6" t="inlineStr">
         <is>
-          <t>Com colarinho colorido</t>
+          <t>750 V</t>
         </is>
       </c>
       <c r="E176" s="6" t="inlineStr">
         <is>
-          <t>Obrigatório em todo borne parafuso</t>
+          <t>24 V de potência — P1 → painel → BTS (6,0 A)</t>
         </is>
       </c>
       <c r="F176" s="7" t="inlineStr"/>
@@ -5070,26 +5014,26 @@
     </row>
     <row r="177">
       <c r="A177" s="9" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B177" s="10" t="inlineStr">
         <is>
-          <t>Alicate de crimpar terminal tubular</t>
+          <t>Cabo flexível 0,75 mm² vermelho/preto</t>
         </is>
       </c>
       <c r="C177" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3 m</t>
         </is>
       </c>
       <c r="D177" s="10" t="inlineStr">
         <is>
-          <t>Tipo quadrado/hexagonal</t>
+          <t>750 V</t>
         </is>
       </c>
       <c r="E177" s="10" t="inlineStr">
         <is>
-          <t>Ferramenta</t>
+          <t>Barramento 24 V (trechos internos) e saída de 12 V do T3 (1,0 A)</t>
         </is>
       </c>
       <c r="F177" s="11" t="inlineStr"/>
@@ -5101,26 +5045,26 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B178" s="6" t="inlineStr">
         <is>
-          <t>Terminal olhal M4</t>
+          <t>Cabo flexível 0,5 mm² (5 cores)</t>
         </is>
       </c>
       <c r="C178" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10 m</t>
         </is>
       </c>
       <c r="D178" s="6" t="inlineStr">
         <is>
-          <t>Amarelo/vermelho</t>
+          <t>750 V</t>
         </is>
       </c>
       <c r="E178" s="6" t="inlineStr">
         <is>
-          <t>Aterramento</t>
+          <t>5 V e derivações do 12 V auxiliar</t>
         </is>
       </c>
       <c r="F178" s="7" t="inlineStr"/>
@@ -5132,26 +5076,26 @@
     </row>
     <row r="179">
       <c r="A179" s="9" t="n">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B179" s="10" t="inlineStr">
         <is>
-          <t>Espaguete termorretrátil (kit)</t>
+          <t>Cabo flexível 0,25 mm² (8 cores)</t>
         </is>
       </c>
       <c r="C179" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15 m</t>
         </is>
       </c>
       <c r="D179" s="10" t="inlineStr">
         <is>
-          <t>Diversas bitolas</t>
+          <t>Sinais</t>
         </is>
       </c>
       <c r="E179" s="10" t="inlineStr">
         <is>
-          <t>Isolação de emendas</t>
+          <t>Sensores, botões, comunicação</t>
         </is>
       </c>
       <c r="F179" s="11" t="inlineStr"/>
@@ -5163,26 +5107,26 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B180" s="6" t="inlineStr">
         <is>
-          <t>Abraçadeiras de nylon 100 mm</t>
+          <t>Cabo par trançado blindado 2×0,25 mm²</t>
         </is>
       </c>
       <c r="C180" s="5" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>2 m</t>
         </is>
       </c>
       <c r="D180" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Blindado, malha aterrada em um ponto</t>
         </is>
       </c>
       <c r="E180" s="6" t="inlineStr">
         <is>
-          <t>Amarração</t>
+          <t>I²C e 1-Wire (trecho câmara → painel)</t>
         </is>
       </c>
       <c r="F180" s="7" t="inlineStr"/>
@@ -5194,11 +5138,11 @@
     </row>
     <row r="181">
       <c r="A181" s="9" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B181" s="10" t="inlineStr">
         <is>
-          <t>Anilhas de identificação de cabo</t>
+          <t>Terminal tubular (ilhós) 0,25 / 0,5 / 1,5 mm²</t>
         </is>
       </c>
       <c r="C181" s="9" t="inlineStr">
@@ -5208,12 +5152,12 @@
       </c>
       <c r="D181" s="10" t="inlineStr">
         <is>
-          <t>Numeradas 0–9</t>
+          <t>Com colarinho colorido</t>
         </is>
       </c>
       <c r="E181" s="10" t="inlineStr">
         <is>
-          <t>Identificação (norma de painel)</t>
+          <t>Obrigatório em todo borne parafuso</t>
         </is>
       </c>
       <c r="F181" s="11" t="inlineStr"/>
@@ -5225,26 +5169,26 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="n">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B182" s="6" t="inlineStr">
         <is>
-          <t>Espiral organizador Ø 8 mm</t>
+          <t>Alicate de crimpar terminal tubular</t>
         </is>
       </c>
       <c r="C182" s="5" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D182" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tipo quadrado/hexagonal</t>
         </is>
       </c>
       <c r="E182" s="6" t="inlineStr">
         <is>
-          <t>Chicote painel → câmara</t>
+          <t>Ferramenta</t>
         </is>
       </c>
       <c r="F182" s="7" t="inlineStr"/>
@@ -5254,11 +5198,35 @@
         <v/>
       </c>
     </row>
-    <row r="183" ht="22" customHeight="1">
-      <c r="A183" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ Itens que NÃO existem mais nesta versão</t>
-        </is>
+    <row r="183">
+      <c r="A183" s="9" t="n">
+        <v>162</v>
+      </c>
+      <c r="B183" s="10" t="inlineStr">
+        <is>
+          <t>Terminal olhal M4</t>
+        </is>
+      </c>
+      <c r="C183" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D183" s="10" t="inlineStr">
+        <is>
+          <t>Amarelo/vermelho</t>
+        </is>
+      </c>
+      <c r="E183" s="10" t="inlineStr">
+        <is>
+          <t>Aterramento</t>
+        </is>
+      </c>
+      <c r="F183" s="11" t="inlineStr"/>
+      <c r="G183" s="12" t="inlineStr"/>
+      <c r="H183" s="12">
+        <f>IF(C183*G183=0,"",C183*G183)</f>
+        <v/>
       </c>
     </row>
     <row r="184">
@@ -5267,12 +5235,24 @@
       </c>
       <c r="B184" s="6" t="inlineStr">
         <is>
-          <t>Fonte ATX 500 W</t>
-        </is>
-      </c>
-      <c r="C184" s="5" t="inlineStr"/>
-      <c r="D184" s="6" t="inlineStr"/>
-      <c r="E184" s="6" t="inlineStr"/>
+          <t>Espaguete termorretrátil (kit)</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D184" s="6" t="inlineStr">
+        <is>
+          <t>Diversas bitolas</t>
+        </is>
+      </c>
+      <c r="E184" s="6" t="inlineStr">
+        <is>
+          <t>Isolação de emendas</t>
+        </is>
+      </c>
       <c r="F184" s="7" t="inlineStr"/>
       <c r="G184" s="8" t="inlineStr"/>
       <c r="H184" s="8">
@@ -5286,12 +5266,24 @@
       </c>
       <c r="B185" s="10" t="inlineStr">
         <is>
-          <t>Jumper PS_ON (verde-preto)</t>
-        </is>
-      </c>
-      <c r="C185" s="9" t="inlineStr"/>
-      <c r="D185" s="10" t="inlineStr"/>
-      <c r="E185" s="10" t="inlineStr"/>
+          <t>Abraçadeiras de nylon 100 mm</t>
+        </is>
+      </c>
+      <c r="C185" s="9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D185" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E185" s="10" t="inlineStr">
+        <is>
+          <t>Amarração</t>
+        </is>
+      </c>
       <c r="F185" s="11" t="inlineStr"/>
       <c r="G185" s="12" t="inlineStr"/>
       <c r="H185" s="12">
@@ -5305,12 +5297,24 @@
       </c>
       <c r="B186" s="6" t="inlineStr">
         <is>
-          <t>Acrílico preto 3 mm (cobertura)</t>
-        </is>
-      </c>
-      <c r="C186" s="5" t="inlineStr"/>
-      <c r="D186" s="6" t="inlineStr"/>
-      <c r="E186" s="6" t="inlineStr"/>
+          <t>Anilhas de identificação de cabo</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>1 kit</t>
+        </is>
+      </c>
+      <c r="D186" s="6" t="inlineStr">
+        <is>
+          <t>Numeradas 0–9</t>
+        </is>
+      </c>
+      <c r="E186" s="6" t="inlineStr">
+        <is>
+          <t>Identificação (norma de painel)</t>
+        </is>
+      </c>
       <c r="F186" s="7" t="inlineStr"/>
       <c r="G186" s="8" t="inlineStr"/>
       <c r="H186" s="8">
@@ -5324,12 +5328,24 @@
       </c>
       <c r="B187" s="10" t="inlineStr">
         <is>
-          <t>Porta simples de acrílico 10 mm</t>
-        </is>
-      </c>
-      <c r="C187" s="9" t="inlineStr"/>
-      <c r="D187" s="10" t="inlineStr"/>
-      <c r="E187" s="10" t="inlineStr"/>
+          <t>Espiral organizador Ø 8 mm</t>
+        </is>
+      </c>
+      <c r="C187" s="9" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="D187" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E187" s="10" t="inlineStr">
+        <is>
+          <t>Chicote painel → câmara</t>
+        </is>
+      </c>
       <c r="F187" s="11" t="inlineStr"/>
       <c r="G187" s="12" t="inlineStr"/>
       <c r="H187" s="12">
@@ -5337,58 +5353,39 @@
         <v/>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="5" t="n">
-        <v>167</v>
-      </c>
-      <c r="B188" s="6" t="inlineStr">
-        <is>
-          <t>XPS 20 mm</t>
-        </is>
-      </c>
-      <c r="C188" s="5" t="inlineStr"/>
-      <c r="D188" s="6" t="inlineStr"/>
-      <c r="E188" s="6" t="inlineStr"/>
-      <c r="F188" s="7" t="inlineStr"/>
-      <c r="G188" s="8" t="inlineStr"/>
-      <c r="H188" s="8">
-        <f>IF(C188*G188=0,"",C188*G188)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="190">
-      <c r="F190" s="13" t="inlineStr">
+    <row r="189">
+      <c r="F189" s="13" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="H190" s="14">
-        <f>SUM(H5:H188)</f>
+      <c r="H189" s="14">
+        <f>SUM(H5:H187)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H188"/>
+  <autoFilter ref="A4:H187"/>
   <mergeCells count="19">
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A98:H98"/>
-    <mergeCell ref="A169:H169"/>
+    <mergeCell ref="A142:H142"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="A183:H183"/>
-    <mergeCell ref="A133:H133"/>
-    <mergeCell ref="A163:H163"/>
+    <mergeCell ref="A88:H88"/>
+    <mergeCell ref="A174:H174"/>
+    <mergeCell ref="A128:H128"/>
+    <mergeCell ref="A164:H164"/>
+    <mergeCell ref="A158:H158"/>
+    <mergeCell ref="A74:H74"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A104:H104"/>
+    <mergeCell ref="A151:H151"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A109:H109"/>
-    <mergeCell ref="A147:H147"/>
-    <mergeCell ref="A156:H156"/>
-    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A44:H44"/>
     <mergeCell ref="A93:H93"/>
+    <mergeCell ref="A58:H58"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5584,7 +5581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -5601,180 +5598,288 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Tensão de entrada</t>
+          <t>Arquitetura de energia</t>
         </is>
       </c>
       <c r="B3" s="20" t="inlineStr">
         <is>
-          <t>127 V CA</t>
+          <t>Potência em 24 V — carga térmica sem conversor</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Barramento de distribuição</t>
+          <t>Tensão de entrada</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
         <is>
-          <t>24 V CC (SELV)</t>
+          <t>127 V CA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Potência instalada (fonte)</t>
+          <t>Barramento de distribuição</t>
         </is>
       </c>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>240 W · 10 A</t>
+          <t>24 V CC (SELV)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>Consumo calculado</t>
+          <t>Potência instalada (fonte)</t>
         </is>
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>≈ 101 W · 4,2 A @ 24 V</t>
+          <t>240 W · 10 A</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Corrente CA de entrada</t>
+          <t>Consumo calculado</t>
         </is>
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>1,44 A</t>
+          <t>≈ 166 W · 6,9 A @ 24 V</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Queda de tensão na linha dos postes</t>
+          <t>Folga da fonte</t>
         </is>
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>0,17 V (0,71 %)</t>
+          <t>1,44× (44 %) — a fonte de 150 W NÃO atende</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Tensões derivadas</t>
+          <t>Corrente CA de entrada</t>
         </is>
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>12,0 V potência · 12,0 V auxiliar · 5,10 V comando · 3,3 V ESP32</t>
+          <t>2,37 A</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>Níveis de proteção</t>
+          <t>Queda de tensão na linha dos postes</t>
         </is>
       </c>
       <c r="B10" s="22" t="inlineStr">
         <is>
-          <t>9 (do disjuntor ao intertravamento por software)</t>
+          <t>0,21 V (0,86 %)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Volume útil da câmara</t>
+          <t>Conversores</t>
         </is>
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>5,0 litros (200 × 100 × 250 mm)</t>
+          <t>2 × LM2596 com display (T2 e T3) · P1 é derivação direta</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Carga térmica calculada</t>
+          <t>Tensões derivadas</t>
         </is>
       </c>
       <c r="B12" s="22" t="inlineStr">
         <is>
-          <t>≈ 9,5 W</t>
+          <t>24,0 V potência (direto) · 12,0 V auxiliar · 5,10 V comando · 3,3 V ESP32</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Capacidade da Peltier a ΔT = 20 K</t>
+          <t>Fusíveis dos ramais</t>
         </is>
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>≈ 30 W (margem de 3,2×)</t>
+          <t>F1 = 10 A · F2 = 2 A · F3 = 2 A (sem F4/F5, sem crowbar)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>Isolamento</t>
+          <t>Níveis de proteção</t>
         </is>
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>XPS 30 mm + barreira de vapor · U = 0,86 W/m²·K</t>
+          <t>5 (do disjuntor ao intertravamento por software)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>Porta</t>
+          <t>Volume útil da câmara</t>
         </is>
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>Dupla · U = 2,42 W/m²·K (não condensa)</t>
+          <t>5,0 litros (200 × 100 × 250 mm)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="21" t="inlineStr">
         <is>
-          <t>Base da maquete</t>
+          <t>Carga térmica calculada</t>
         </is>
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>900 × 500 mm · escala cenográfica 1:50</t>
+          <t>≈ 9,5 W</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
         <is>
+          <t>Refrigeração</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>2 × TEC1-12706 EM SÉRIE · 24 V · 6,0 A · 144 W</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Capacidade das Peltier a ΔT = 20 K</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>≈ 60 W (margem de 6,3×)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Dissipação no lado quente</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>≈ 200 W — 2 conjuntos dissipador + cooler 80 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>Aquecimento</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>PTC cerâmico de 24 V · 60 W · 2,5 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>Isolamento</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>XPS 30 mm + barreira de vapor · U = 0,86 W/m²·K</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Porta</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Dupla · U = 2,42 W/m²·K (não condensa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Base da maquete</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>1500 × 500 mm · escala cenográfica 1:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
           <t>Painel</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>400 × 500 × 200 mm · 3 trilhos DIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Componentes discretos</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>6 + 1 CI ULN2803 na PI-1 · 2 nos BTS7960 · 4 nos postes da maquete</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Sinalização</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>4 sinaleiros 22 mm de 24 V (via ULN2803) · 4 LEDs brancos de 5 V na maquete</t>
         </is>
       </c>
     </row>

</xml_diff>